<commit_message>
The third edition of the product backlog with prioritization has been translated into English, and adjustments have been made to the wording
</commit_message>
<xml_diff>
--- a/Product_Backlog.xlsx
+++ b/Product_Backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java项目\EBU6304-Group17\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F207875-0B29-42BA-86B0-462115AFD789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{559A696C-3E3C-471B-9159-FD89550A16CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="224">
   <si>
     <t>Story ID</t>
   </si>
@@ -52,611 +52,85 @@
     <t>P0-001</t>
   </si>
   <si>
-    <t>创建个人助教申请档案</t>
-  </si>
-  <si>
-    <t>作为一名应聘者，我想要填写并保存我的个人基础信息（姓名、学号、所属专业、联系电话、邮箱、可任职时间段、个人基础技能），以便我能够提交助教岗位申请。</t>
-  </si>
-  <si>
     <t>P0</t>
   </si>
   <si>
-    <t>1. 应聘者可进入档案创建页面，填写所有必填字段
-2. 系统对空值输入进行校验并提示
-3. 填写完成后，信息可本地持久化存储为 JSON 格式
-4. 同一学号不可重复创建档案</t>
-  </si>
-  <si>
-    <t>JSON 存储，无数据库</t>
-  </si>
-  <si>
     <t>P0-002</t>
   </si>
   <si>
-    <t>查看可申请助教岗位列表</t>
-  </si>
-  <si>
-    <t>作为一名应聘者，我想要查看所有可申请的助教岗位信息，以便我选择合适的岗位进行申请。</t>
-  </si>
-  <si>
-    <t>1. 应聘者登录后可进入岗位列表页面
-2. 页面展示岗位核心信息：岗位名称、所属课程 / 活动、招聘人数、任职要求、申请截止时间、发布人
-3. 已截止岗位标注为不可申请状态</t>
-  </si>
-  <si>
     <t>P0-003</t>
   </si>
   <si>
-    <t>提交助教岗位申请</t>
-  </si>
-  <si>
-    <t>作为一名应聘者，我想要选择目标岗位并提交我的申请，以便课程组织者能够查看我的应聘信息。</t>
-  </si>
-  <si>
-    <t>1. 应聘者可在岗位详情页点击申请按钮
-2. 系统校验该应聘者是否已对同一岗位提交过申请，重复申请则提示禁止
-3. 申请提交后生成唯一申请记录，状态为「审核中」
-4. 申请信息与应聘者档案关联存储</t>
-  </si>
-  <si>
     <t>P0-004</t>
   </si>
   <si>
-    <t>查看个人申请状态</t>
-  </si>
-  <si>
-    <t>作为一名应聘者，我想要查询我所有的申请记录及状态，以便了解我的应聘进展。</t>
-  </si>
-  <si>
-    <t>1. 应聘者可进入申请记录页面，查看所有申请记录
-2. 每条记录展示岗位名称、申请时间、当前状态（已提交 / 审核中 / 通过 / 未通过）
-3. 状态与课程组织者的审核操作实时同步</t>
-  </si>
-  <si>
     <t>P0-005</t>
   </si>
   <si>
-    <t>发布助教岗位</t>
-  </si>
-  <si>
-    <t>作为一名课程组织者（MO），我想要填写并发布助教岗位信息，以便应聘者能够看到并申请该岗位</t>
-  </si>
-  <si>
-    <t>1. MO 可进入岗位发布页面，填写岗位基础信息
-2. 发布后岗位自动上线至公开岗位列表
-3. 可设置申请截止时间，到达时间后岗位自动不可申请</t>
-  </si>
-  <si>
     <t>P0-006</t>
   </si>
   <si>
-    <t>查看本岗位应聘者列表</t>
-  </si>
-  <si>
-    <t>作为一名课程组织者（MO），我想要查看我发布岗位的所有应聘者信息，以便进行审核。</t>
-  </si>
-  <si>
-    <t>1. MO 可进入本人发布的岗位详情页
-2. 页面展示对应岗位的所有应聘者基础档案信息、申请提交时间
-3. 仅展示当前登录 MO 发布岗位的应聘者</t>
-  </si>
-  <si>
     <t>P0-007</t>
   </si>
   <si>
-    <t>单条审核应聘者申请</t>
-  </si>
-  <si>
-    <t>作为一名课程组织者（MO），我想要对单个应聘者的申请标记通过 / 未通过，以便完成应聘筛选并同步状态给应聘者。</t>
-  </si>
-  <si>
-    <t>1. MO 可在应聘者列表中对单条申请选择「通过」或「未通过」
-2. 审核操作后，应聘者的申请状态自动更新
-3. 状态变更同步至应聘者的申请记录页面</t>
-  </si>
-  <si>
     <t>P0-009</t>
   </si>
   <si>
-    <t>角色登录验证</t>
-  </si>
-  <si>
-    <t>1. 用户可进入登录页面，输入账号密码
-2. 系统验证账号密码有效性，验证失败则提示
-3. 不同角色登录后跳转至对应操作界面（应聘者 / MO/ 管理员）
-4. 登录信息可本地存储</t>
-  </si>
-  <si>
-    <t>核心数据持久化</t>
-  </si>
-  <si>
-    <t>作为一名系统开发者，我想要实现用户档案、岗位信息、申请记录的增删改查并持久化存储，以便保证数据不丢失。</t>
-  </si>
-  <si>
-    <t>1. 所有用户档案、岗位信息、申请记录均支持增删改查操作
-2. 数据存储为JSON 格式
-3. 数据读取和写入无异常</t>
-  </si>
-  <si>
     <t>P0-011</t>
   </si>
   <si>
-    <t>基础错误处理</t>
-  </si>
-  <si>
-    <t>1. 对空值输入、重复申请、已截止岗位申请、无效账号登录等操作给出文字提示
-2. 提示信息清晰易懂，指导用户修正操作
-3. 异常操作不会导致系统崩溃</t>
-  </si>
-  <si>
     <t>P0-012</t>
   </si>
   <si>
-    <t>核心功能界面交互</t>
-  </si>
-  <si>
-    <t>1. 实现登录页、档案创建页、岗位列表页、申请审核页等核心界面
-2. 界面导航清晰，操作按钮布局合理
-3. 核心操作流程无阻断，跳转顺畅</t>
-  </si>
-  <si>
-    <t>中/低保真原型基础交互</t>
-  </si>
-  <si>
     <t>P1-001</t>
   </si>
   <si>
-    <t>编辑个人申请档案</t>
-  </si>
-  <si>
-    <t>作为一名应聘者，我想要在未提交申请时修改我的档案信息，以便更新我的个人情况。</t>
-  </si>
-  <si>
     <t>P1</t>
   </si>
   <si>
-    <t>1. 未提交任何岗位申请的应聘者可编辑档案信息
-2. 已提交申请的应聘者仅可修改非申请关联信息
-3. 编辑后信息自动更新存储</t>
-  </si>
-  <si>
     <t>P1-002</t>
   </si>
   <si>
-    <t>按条件筛选岗位</t>
-  </si>
-  <si>
-    <t>1. 岗位列表页提供筛选条件输入框
-2. 支持按课程名称 / 活动类型、可任职时间、招聘人数筛选
-3. 筛选后页面实时更新展示符合条件的岗位</t>
-  </si>
-  <si>
-    <t>撤回未审核申请</t>
-  </si>
-  <si>
-    <t>作为一名应聘者，我想要撤回状态为「审核中」的申请，以便重新选择或修改申请。</t>
-  </si>
-  <si>
-    <t>1. 仅状态为「审核中」的申请可撤回
-2. 撤回后申请记录状态更新为「已撤回」
-3. 岗位可重新被该应聘者申请</t>
-  </si>
-  <si>
-    <t>上传个人简历</t>
-  </si>
-  <si>
-    <t>作为一名应聘者，我想要上传纯文本 / Word 格式简历，以便课程组织者更全面了解我的能力。</t>
-  </si>
-  <si>
-    <t>1. 应聘者可在档案页上传简历文件
-2. 系统存储简历文件路径至档案
-3. MO 可查看应聘者上传的简历内容</t>
-  </si>
-  <si>
-    <t>存储文件路径，不直接存储文件内容</t>
-  </si>
-  <si>
-    <t>申请记录详情查看</t>
-  </si>
-  <si>
-    <t>多条件筛选应聘者</t>
-  </si>
-  <si>
-    <t>作为一名课程组织者（MO），我想要按专业、可任职时间等条件筛选应聘者，以便快速找到符合要求的候选人。</t>
-  </si>
-  <si>
-    <t>1. 应聘者列表页提供筛选条件输入框
-2. 支持按专业、可任职时间、基础技能筛选
-3. 筛选后页面实时更新展示符合条件的应聘者</t>
-  </si>
-  <si>
-    <t>批量审核应聘者申请</t>
-  </si>
-  <si>
-    <t>作为一名课程组织者（MO），我想要批量标记多个应聘者的申请状态，以便提升审核效率。</t>
-  </si>
-  <si>
-    <t>1. MO 可在应聘者列表中勾选多条申请
-2. 可对勾选的申请批量选择「通过」或「未通过」
-3. 批量操作后所有选中申请的状态同步更新</t>
-  </si>
-  <si>
-    <t>导出应聘者列表</t>
-  </si>
-  <si>
-    <t>作为一名课程组织者（MO），我想要将本岗位应聘者信息导出为 Excel 格式，以便线下查看和统计。</t>
-  </si>
-  <si>
-    <t>1. MO 可在应聘者列表页点击导出按钮
-2. 导出文件为 Excel 格式，包含应聘者核心信息
-3. 导出文件可正常打开查看</t>
-  </si>
-  <si>
-    <t>本账号岗位统计</t>
-  </si>
-  <si>
-    <t>作为一名课程组织者（MO），我想要查看我发布的所有岗位的核心数据，以便了解招聘进度。</t>
-  </si>
-  <si>
-    <t>1. MO 可进入岗位统计页面
-2. 展示本人发布岗位的状态（已发布 / 已下架 / 已截止）、申请人数、通过人数
-3. 数据统计准确实时</t>
-  </si>
-  <si>
-    <t>基础账号管理</t>
-  </si>
-  <si>
-    <t>作为一名系统管理员，我想要重置 MO / 应聘者的密码或删除无效账号，以便维护账号安全。</t>
-  </si>
-  <si>
-    <t>1. 管理员可重置任意用户的账号密码
-2. 可删除无效 / 过期账号
-3. 操作后账号状态同步更新</t>
-  </si>
-  <si>
-    <t>全局岗位查看</t>
-  </si>
-  <si>
-    <t>岗位时间提醒</t>
-  </si>
-  <si>
-    <t>作为一名应聘者，我想要在查看岗位时看到截止时间提醒，以便及时申请。</t>
-  </si>
-  <si>
-    <t>1. 距离截止＜24 小时的岗位标注「即将截止」
-2. 已截止岗位标注「不可申请」
-3. 提醒标识清晰可见</t>
-  </si>
-  <si>
-    <t>分页展示列表</t>
-  </si>
-  <si>
-    <t>1. 岗位列表、应聘者列表、申请记录列表实现分页
-2. 每页展示固定数量数据，支持翻页操作
-3. 分页导航清晰易用</t>
-  </si>
-  <si>
-    <t>关键操作日志</t>
-  </si>
-  <si>
-    <t>作为一名系统管理员，我想要记录关键操作并可查看日志，以便追溯操作历史。</t>
-  </si>
-  <si>
-    <t>1. 记录发布岗位、提交申请、审核申请、账号登录等操作
-2. 日志存储为文本文件
-3. 管理员可查看日志内容</t>
-  </si>
-  <si>
     <t>P2-001</t>
   </si>
   <si>
-    <t>收藏意向岗位</t>
-  </si>
-  <si>
-    <t>作为一名应聘者，我想要收藏感兴趣的岗位，以便后续快速查看和申请。</t>
-  </si>
-  <si>
     <t>P2</t>
   </si>
   <si>
-    <t>1. 应聘者可在岗位列表 / 详情页点击收藏按钮
-2. 收藏岗位单独展示在收藏列表页
-3. 可取消收藏</t>
-  </si>
-  <si>
     <t>P2-002</t>
   </si>
   <si>
-    <t>申请状态本地提醒</t>
-  </si>
-  <si>
-    <t>作为一名应聘者，我想要在申请状态变更时收到提示，以便及时了解应聘结果。</t>
-  </si>
-  <si>
-    <t>1. 登录后若申请状态变更，弹出消息提示
-2. 提示内容包含岗位名称和状态变更结果
-3. 可关闭提示</t>
-  </si>
-  <si>
-    <t>本地提示，无短信 / 邮件推送</t>
-  </si>
-  <si>
-    <t>查看个人申请历史</t>
-  </si>
-  <si>
-    <t>作为一名应聘者，我想要按时间筛选我的所有申请记录，以便回顾应聘历史。</t>
-  </si>
-  <si>
-    <t>1. 申请记录页支持按时间筛选
-2. 展示所有申请记录（含已撤回、未通过）
-3. 筛选后列表实时更新</t>
-  </si>
-  <si>
-    <t>档案信息导出</t>
-  </si>
-  <si>
-    <t>作为一名应聘者，我想要将我的档案信息导出为JSON 格式，以便线下备份。</t>
-  </si>
-  <si>
-    <t>1. 应聘者可在档案页点击导出按钮
-2. 导出文件为JSON 格式，包含所有档案信息
-3. 导出文件可正常打开查看</t>
-  </si>
-  <si>
-    <t>是否选用JSON格式待讨论</t>
-  </si>
-  <si>
-    <t>设定岗位技能要求</t>
-  </si>
-  <si>
-    <t>作为一名课程组织者（MO），我想要在发布岗位时添加具体技能要求，以便精准匹配招聘需求。</t>
-  </si>
-  <si>
-    <t>1. 岗位发布页可添加技能要求字段
-2. 技能要求可多选或输入
-3. 技能要求展示在岗位详情页</t>
-  </si>
-  <si>
-    <t>添加审核评语</t>
-  </si>
-  <si>
-    <t>作为一名课程组织者（MO），我想要在审核时填写评语，以便向应聘者说明审核原因。</t>
-  </si>
-  <si>
-    <t>1. 审核时可输入文字评语
-2. 评语同步至应聘者的申请记录详情页
-3. 评语长度有限制（如最多 200 字</t>
-  </si>
-  <si>
-    <t>岗位截止时间自动下架</t>
-  </si>
-  <si>
-    <t>作为一名课程组织者（MO），我想要岗位在到达截止时间后自动下架，以便避免接收过期申请。</t>
-  </si>
-  <si>
-    <t>1. 到达申请截止时间的岗位自动下架
-2. 下架后从公开列表隐藏，不可提交新申请
-3. 已提交的申请仍可被审核</t>
-  </si>
-  <si>
-    <t>查看 TA 任职基础信息</t>
-  </si>
-  <si>
-    <t>作为一名课程组织者（MO），我想要查看应聘者的过往助教任职经历，以便辅助审核决策。</t>
-  </si>
-  <si>
-    <t>1. 应聘者档案中包含过往任职经历字段
-2. MO 在审核时可查看该信息
-3. 信息展示清晰</t>
-  </si>
-  <si>
-    <t>工作负荷阈值预警</t>
-  </si>
-  <si>
-    <t>作为一名系统管理员，我想要设定 TA 工作负荷阈值，以便在 TA 负荷过高时收到预警。</t>
-  </si>
-  <si>
-    <t>1. 管理员可设定阈值（如单学期最多 3 个岗位）
-2. TA 任职数接近 / 超过阈值时，系统给出文字预警
-3. 预警展示在工作负荷页面</t>
-  </si>
-  <si>
-    <t>全院招聘数据统计</t>
-  </si>
-  <si>
-    <t>作为一名系统管理员，我想要统计全院的招聘数据，以便辅助学院管理决策。</t>
-  </si>
-  <si>
-    <t>1. 统计各课程 / 活动的招聘完成率、TA 任职分布、各 MO 招聘进度
-2. 以表格形式展示
-3. 数据统计准确实时</t>
-  </si>
-  <si>
-    <t>全局数据导出</t>
-  </si>
-  <si>
-    <t>作为一名系统管理员，我想要将全院核心数据导出为 CSV 格式，以便线下分析。</t>
-  </si>
-  <si>
-    <t>1. 管理员可导出岗位信息、TA 任职信息、招聘统计数据
-2. 导出文件为 CSV 格式
-3. 导出文件可正常打开查看</t>
-  </si>
-  <si>
-    <t>操作权限基础管控</t>
-  </si>
-  <si>
-    <t>作为一名系统管理员，我想要限制 MO 仅能操作本人发布的岗位，以便保障数据安全。</t>
-  </si>
-  <si>
-    <t>1. MO 仅能查看 / 操作本人发布的岗位
-2. 禁止跨账号查看 / 审核其他 MO 的岗位应聘者
-3. 权限校验在操作前执行</t>
-  </si>
-  <si>
-    <t>数据手动备份与恢复</t>
-  </si>
-  <si>
-    <t>作为一名系统管理员，我想要手动备份和恢复系统数据，以便防止数据丢失。</t>
-  </si>
-  <si>
-    <t>1. 管理员可备份所有系统数据（用户、岗位、申请记录）
-2. 备份文件可恢复至系统
-3. 备份 / 恢复操作有明确提示</t>
-  </si>
-  <si>
-    <t>界面交互优化</t>
-  </si>
-  <si>
-    <t>作为一名系统用户，我想要使用更友好的界面，以便提升操作体验。</t>
-  </si>
-  <si>
-    <t>1. 完善界面导航、弹窗提示、操作按钮布局
-2. 界面符合中保真原型标准
-3. 操作流程更顺畅</t>
-  </si>
-  <si>
-    <t>中英文双语界面</t>
-  </si>
-  <si>
-    <t>作为一名国际学院用户，我想要切换中英文界面，以便适配国际化使用场景。</t>
-  </si>
-  <si>
-    <t>1. 系统支持中文 / 英文界面切换
-2. 核心文字均有双语版本
-3. 切换后界面实时更新</t>
-  </si>
-  <si>
     <t>P3-001</t>
   </si>
   <si>
-    <t>个人技能与岗位匹配度提示</t>
-  </si>
-  <si>
-    <t>作为一名应聘者，我想要看到我的技能与岗位的匹配度评分，以便辅助选择岗位。</t>
-  </si>
-  <si>
     <t>P3</t>
   </si>
   <si>
-    <t>1. 岗位详情页展示匹配度评分（百分比）
-2. 评分基于应聘者技能与岗位技能要求计算
-3. 评分逻辑可解释</t>
-  </si>
-  <si>
-    <t>AI 增值功能，可选实现</t>
-  </si>
-  <si>
     <t>P3-002</t>
   </si>
   <si>
-    <t>技能短板识别提示</t>
-  </si>
-  <si>
-    <t>作为一名应聘者，我想要在申请后看到我的技能短板及提升建议，以便针对性提升能力。</t>
-  </si>
-  <si>
-    <t>1. 申请后系统对比岗位要求，指出缺失技能
-2. 给出基础提升建议
-3. 提示内容清晰易懂</t>
-  </si>
-  <si>
     <t>P3-003</t>
   </si>
   <si>
-    <t>应聘者技能智能筛选</t>
-  </si>
-  <si>
-    <t>作为一名课程组织者（MO），我想要系统自动筛选高匹配度应聘者并优先展示，以便提升筛选效率。</t>
-  </si>
-  <si>
-    <t>1. 应聘者列表按匹配度排序，高匹配度优先展示
-2. 匹配度基于岗位技能要求计算
-3. 可手动调整排序</t>
-  </si>
-  <si>
     <t>P3-004</t>
   </si>
   <si>
-    <t>简历关键词提取</t>
-  </si>
-  <si>
-    <t>作为一名课程组织者（MO），我想要系统自动提取简历核心关键词，以便快速了解应聘者能力。</t>
-  </si>
-  <si>
-    <t>1. 系统从简历中提取核心技能、任职经历等关键词
-2. 关键词展示在应聘者信息页
-3. 提取结果可人工核验</t>
-  </si>
-  <si>
     <t>P3-005</t>
   </si>
   <si>
-    <t>TA 工作负荷均衡分配建议</t>
-  </si>
-  <si>
-    <t>作为一名系统管理员，我想要获取 TA 岗位分配优化建议，以便均衡工作负荷。</t>
-  </si>
-  <si>
-    <t>1. 系统基于当前 TA 负荷给出分配建议
-2. 建议可人工查看和修改
-3. 建议逻辑可解释</t>
-  </si>
-  <si>
     <t>P3-006</t>
   </si>
   <si>
-    <t>招聘需求智能统计</t>
-  </si>
-  <si>
-    <t>作为一名系统管理员，我想要获取各课程 / 活动的助教招聘人数参考建议，以便辅助制定计划。</t>
-  </si>
-  <si>
-    <t>1. 基于过往数据给出招聘人数参考
-2. 参考可人工调整
-3. 统计逻辑可解释</t>
-  </si>
-  <si>
     <t>P3-007</t>
   </si>
   <si>
-    <t>AI 匹配逻辑可配置</t>
-  </si>
-  <si>
-    <t>作为一名系统管理员，我想要调整岗位技能匹配的权重，以便让匹配结果更贴合实际需求。</t>
-  </si>
-  <si>
-    <t>1. 可配置专业技能、任职经历等权重
-2. 配置后匹配度计算实时更新
-3. 配置界面清晰易用</t>
-  </si>
-  <si>
     <t>P3-008</t>
   </si>
   <si>
-    <t>AI 结果人工核验</t>
-  </si>
-  <si>
-    <t>作为一名系统用户，我想要核验 AI 生成的结果，以便避免逻辑错误。</t>
-  </si>
-  <si>
-    <t>1. 所有 AI 生成结果支持人工查看
-2. 可手动修改 AI 结果
-3. 修改后结果覆盖 AI 生成内容</t>
-  </si>
-  <si>
-    <t>导出格式待定</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Estimation/day</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>不确定的</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>P2-003</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -677,44 +151,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>编辑</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>已发布岗位</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>仅未截止且无应聘者申请的岗位可编辑</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>P0-013</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -727,10 +163,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>下架已发布岗位</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>P1-003</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -819,155 +251,696 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>作为一名应聘者 / 课程组织者 (MO)/ 系统管理员，我想要在操作异常时收到明确提示，以便了解操作失败的原因。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>作为一名应聘者 / 课程组织者 (MO)/ 系统管理员，我想要使用顺畅的界面完成核心操作，以便提升使用体验。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">
-2. 可手动下架岗位，下架后从公开列表隐藏
-3. 下架岗位不可再接收新申请</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>应聘者可点击申请记录进入详情页
-2. 详情页展示岗位详情、申请时间、审核人、审核意见（若有）
-3. 信息展示完整清晰</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>作为一名课程组织者（MO），我想要编辑未截止且无应聘者的岗位信息，以便调整招聘需求。</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>作为一名系统管理员，我想要查看所有 MO 和应聘者的个人信息，以便掌握全院招聘进度。</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>管理员可进入全局查看列表（可以查看所有用户）
-2. 展示用户的所有信息，包括个人信息，TA：应聘的信息，MO：收到的申请，等信息</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>作为一名应聘者 / 课程组织者 (MO)/ 系统管理员，我想要在列表数据过多时看到分页展示，以便提升浏览体验。</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>优先度升到P1</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>下降到P2</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>优先级下降到P2</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>作为一名应聘者 / 课程组织者 (MO)/ 系统管理员，我想要通过账号密码登录系统，以便进入对应角色的操作界面。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>作为一名课程组织者（MO），我想要下架未截止的岗位信息，以便调整招聘需求。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>作为一名应聘者，我想要按课程名称 / 可任职时间等条件筛选岗位，以便快速找到合适的岗位。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>作为一名应聘者，我想要查看申请记录的完整信息，以便了解申请的详细情况。</t>
+    <t>Create a personal teaching assistant application file</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>View the list of teaching assistant positions you can apply for</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Submit an application for a teaching assistant position</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Check the status of your application</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Release teaching assistant positions</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. MOs can enter the job posting page and fill in the basic information of the position
+2. After the posting, the job will be automatically launched to the public job list
+3. You can set the application deadline, and the position will automatically not be able to apply after the time is reached</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Single review of applicants' applications</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. MO can select "Passed" or "Unsuccessful" for a single application in the list of applicants
+2. After reviewing the operation, the applicant's application status will be updated automatically
+3. The status change is synced to the applicant's application history page</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Role login verification</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Users can enter the login page and enter their account password
+2. The system verifies the validity of the account password, and prompts if the verification fails
+3. After logging in to different roles, you will be redirected to the corresponding operation interface (Applicant / MO / Administrator)
+4. Login information can be stored locally</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Basic error handling</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Text prompts are given for operations such as null value input, repeated application, closed job application, and invalid account login
+2. The prompt information is clear and easy to understand, guiding users to correct the operation
+3. Abnormal operations will not cause system crashes</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Core function interface interaction</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Implement core interfaces such as login page, file creation page, job list page, and application review page
+2. The interface is clear and the operation buttons are reasonably laid out
+3. The core operation process is uninterrupted and the jump is smooth</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>JSON storage, no database</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Medium/low-fidelity prototype base interaction</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Withdraw unreviewed applications</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Removed posted posts</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Only applications with a status of "Under Review" can be withdrawn
+2. Update the status of the application record to "Withdrawn" after withdrawal
+3. The position can be re-applied by the applicant</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. You can manually remove the post and hide it from the public list after removal
+2. No new applications will be accepted for the removed positions</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Edit your personal application file</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Position selection according to conditions</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. The job list page provides a filter input box
+2. Support filtering by course name/activity type, available hours, and number of recruits
+3. After filtering, the page is updated in real time to display eligible positions</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Upload your resume</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Store the file path and do not store the file content directly</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Please check the details of the application record</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Editor posted jobs</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Only positions that have not been closed and have not been applied for by applicants can be edited</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Review applicant applications in bulk</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Statistics of this account</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. MO can enter the job statistics page
+2. Display the status of the posted position (published/removed/closed), the number of applicants, and the number of passes
+3. Accurate and real-time data statistics</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Global post view</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Administrators can enter the global view list (all users can be viewed)
+2. Display all information of the user, including personal information, TA: application information, MO: application received, etc</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Basic account management</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Administrators can reset the account password of any user
+2. Invalid / expired accounts can be deleted
+3. The account status will be updated synchronously after the operation</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Paginated display list</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Job list, applicant list, and application record list are paginated
+2. Each page displays a fixed amount of data and supports page turning operations
+3. Pagination navigation is clear and easy to use</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Key operation logs</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Record the posting of positions, submitting applications, reviewing applications, account logins, etc
+2. The logs are stored as text files
+3. Administrators can view the log contents</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>View individual application history</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. The application record page supports filtering by time
+2. Display all application records (including withdrawn and unsuccessful)
+3. The list is updated in real time after filtering</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Collect the intended position</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Local alerts on application status</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. If the application status changes after logging in, a pop-up message will appear
+2. The prompt content includes the job title and status change results
+3. Prompts can be turned off</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Local prompts, no SMS/email push</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>File information export</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Whether to choose JSON format is to be discussed</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Set job skill requirements</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. You can add a skill requirement field to the job posting page
+2. Skill requirements can be selected or entered
+3. Skill requirements are displayed on the job details page</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Add review comments</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. You can enter text comments during the review
+2. Comments are synchronized to the applicant's application record details page
+3. There is a limit to the length of the comment (e.g. up to 200 words).</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>The job cut-off time will be automatically removed from the shelves</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Positions that have reached the application deadline will be automatically removed
+2. After removal, it will be hidden from the public list and new applications cannot be submitted
+3. Submitted applications can still be reviewed</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>View the TA Job Fundamentals information</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Workload threshold alerts</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Administrators can set thresholds (e.g. up to 3 positions in a single semester)
+2. When the number of TA positions approaches/exceeds the threshold, the system will give a text warning
+3. Alerts are displayed on the Workload page</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Statistics of recruitment data of the whole hospital</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Statistics on the recruitment completion rate, TA job distribution, and recruitment progress of each MO for each course/activity
+2. Present in a table
+3. Accurate and real-time data statistics</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Global data export</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Administrators can export job information, TA job information, and recruitment statistics
+2. Export the file in CSV format
+3. The exported file can be opened and viewed normally</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Export format TBD</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Basic control of operation permissions</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. MO can only view/operate the posts posted by the MO
+2. It is prohibited to view/review applicants for other MO positions across accounts
+3. Permission verification is performed before operation</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Manually backup and restore data</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Administrators can back up all system data (users, positions, application records)
+2. The backup file can be restored to the system
+3. There are clear prompts for backup/restore operations</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Interface interaction optimization</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Improve the interface navigation, pop-up prompts, and operation button layout
+2. The interface complies with the medium-fidelity prototype standard
+3. Smoother operation process</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Bilingual interface in Chinese and English</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. The system supports switching between Chinese and English interfaces
+2. The core text is bilingual
+3. The interface is updated in real time after switching</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Job time reminder</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Positions marked with "Coming soon" &lt; 24 hours from the deadline
+2. Closed positions marked as "Not Applicable"
+3. The reminder sign is clearly visible</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Tips on the matching degree of personal skills and positions</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AI value-added functions, optionally implemented</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Skill shortcomings identification tips</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. After applying, the system compares the job requirements and points out the missing skills
+2. Give suggestions for basic improvement
+3. The prompt content is clear and easy to understand</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Resume keyword extraction</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. The system extracts key words such as core skills and work experience from the resume
+2. Keywords are displayed on the applicant's information page
+3. The extraction results can be manually verified</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TA workload equalization recommendation</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. The system gives an allocation recommendation based on the current TA load
+2. Suggestions can be viewed and modified manually
+3. Suggest logic that is explainable</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Intelligent statistics of recruitment demand</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Give a reference to the number of recruits based on past data
+2. References can be adjusted manually
+3. Statistical logic is explainable</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AI matching logic is configurable</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. Weights such as professional skills and work experience can be configured
+2. The matching calculation is updated in real time after configuration
+3. The configuration interface is clear and easy to use</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AI results are manually verified</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. All AI-generated results support human viewing
+2. AI results can be modified manually
+3. The modified result overlays the AI-generated content</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Uncertain</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Core data persistence</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a system developer, I want to add and delete user files, job information, and application records, and store them persistently to ensure that data is not lost.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. All user files, job information, and application records can be added, deleted, modified, and checked
+2. The data is stored in JSON format
+3. Data reading and writing without abnormalities</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1. TAs can go to the profile creation page and fill in all required fields
+2. The system checks and prompts the null input
+3. Once completed, the information can be persistently stored in JSON format locally
+4. The same student number cannot create files repeatedly</t>
+  </si>
+  <si>
+    <t>As a TA, I want to view all the available teaching assistant positions so that I can choose the right position to apply.</t>
+  </si>
+  <si>
+    <t>1. TAs can enter the job list page after logging in
+2. The page displays the core information of the position: job title, course/activity, number of recruits, job requirements, application deadline, and publisher
+3. Closed positions are marked as unappliable</t>
+  </si>
+  <si>
+    <t>1. TAs can click the application button on the job details page
+2. The system checks whether the applicant has submitted an application for the same position, and repeated applications are prohibited
+3. After the application is submitted, a unique application record is generated with the status "Under Review"
+4. The application information is stored in association with the applicant's file</t>
+  </si>
+  <si>
+    <t>1. TAs can go to the application history page to view all application records
+2. Each record shows the job title, application time, and current status (submitted/under review/passed/failed)
+3. The status is synchronized in real-time with the course organizer's review actions</t>
+  </si>
+  <si>
+    <t>View the list of TAs for this position</t>
+  </si>
+  <si>
+    <t>1. MO can enter the job details page posted by me
+2. The page displays the basic file information of all applicants for the corresponding position and the application submission time
+3. Only TAs who are currently logged in to the MO posting position will be displayed</t>
+  </si>
+  <si>
+    <t>1. TAs who have not submitted any job applications can edit their file information
+2. TAs who have submitted an application can only modify the non-application related information
+3. The information is automatically updated and stored after editing</t>
+  </si>
+  <si>
+    <t>1. TAs can upload resume files on the profile page
+2. The system stores the resume file path to the file
+3. MO can view the content of the resume uploaded by the TA</t>
+  </si>
+  <si>
+    <t>As a TA, I want to see the full information on the application record so that I can understand the details of the application.</t>
+  </si>
+  <si>
+    <t>1. TAs can click on the application record to enter the details page
+2. The details page displays the job details, application time, reviewer, and review opinions (if any)
+3. The information display is complete and clear</t>
+  </si>
+  <si>
+    <t>TAs are screened with multiple conditions</t>
+  </si>
+  <si>
+    <t>1. The TA list page provides a filter input box
+2. Support screening by major, available working hours, and basic skills
+3. After filtering, the page will update in real time to show qualified TAs</t>
+  </si>
+  <si>
+    <t>1. MO can tick multiple applications from the list of TAs
+2. You can select "Passed" or "Rejected" in batches for the checked applications.
+3. After the batch operation, the status of all selected applications is updated synchronously</t>
+  </si>
+  <si>
+    <t>As a TA, I want to sift through all my application records by time so that I can review my application history.</t>
+  </si>
+  <si>
+    <t>As a TA, I want to save the positions I am interested in so that I can quickly view and apply for them later.</t>
+  </si>
+  <si>
+    <t>1. TAs can click the Favorite button on the job list/details page
+2. Favorite positions are displayed separately on the collection list page
+3. You can cancel your collection</t>
+  </si>
+  <si>
+    <t>1. TAs can click the export button on the profile page
+2. The export file is in JSON format and contains all the archive information
+3. The exported file can be opened and viewed normally</t>
+  </si>
+  <si>
+    <t>1. TA profiles include past employment fields
+2. The MO can view this information at the time of the review
+3. Clear information presentation</t>
+  </si>
+  <si>
+    <t>As a TA, I want to see a deadline reminder when I check a position so that I can apply in time.</t>
+  </si>
+  <si>
+    <t>Export the list of TAs</t>
+  </si>
+  <si>
+    <t>1. MO can be clicked on the export button on the applicant list page
+2. The export file is in Excel format and contains the TA's core information
+3. The exported file can be opened and viewed normally</t>
+  </si>
+  <si>
+    <t>1. Job details page display match score (percentage)
+2. Scoring is calculated based on the TA's skills and job skills
+3. The scoring logic is explainable</t>
+  </si>
+  <si>
+    <t>As a TA, I want to see my skills shortcomings and suggestions for improvement after applying, so that I can improve my abilities in a targeted manner.</t>
+  </si>
+  <si>
+    <t>Intelligent screening of TA skills</t>
+  </si>
+  <si>
+    <t>1. The list of TAs is sorted by match, and high matching is prioritized
+2. The matching degree is calculated based on the job skill requirements
+3. Manually adjust the sorting</t>
+  </si>
+  <si>
+    <t>As a MO, I want to fill out and post the teaching assistant position so that TAs can see and apply for the position</t>
+  </si>
+  <si>
+    <t>As a MO, I want to take down open job postings so I can adjust my hiring needs.</t>
+  </si>
+  <si>
+    <t>As a MO, I want to edit the information for unclosed and unqualified positions so that I can adjust my hiring needs.</t>
+  </si>
+  <si>
+    <t>As a MO, I want to screen TAs by major, availability, etc., so that I can quickly find TAs who meet the requirements.</t>
+  </si>
+  <si>
+    <t>As a MO, I want positions to be automatically removed when the deadline is reached so that I don't receive late applications.</t>
+  </si>
+  <si>
+    <t>As a TA/MO/ Admin, I want to be clearly alerted when an operation is abnormal so that I can understand why the operation failed.</t>
+  </si>
+  <si>
+    <t>As a Admin, I want to set TA workload thresholds so that I can be alerted when TA is overloaded.</t>
+  </si>
+  <si>
+    <t>As a Admin, I want to manually back up and restore system data so that data loss is prevented.</t>
+  </si>
+  <si>
+    <t>As a TA, I want to fill in and save my personal basic information (name, student number, major, contact number, email, available time period, personal basic skills) so that I can submit my application for the teaching assistant position.</t>
+  </si>
+  <si>
+    <t>As a TA, I want to select the target position and submit my application so that the course organizer can view my application.</t>
+  </si>
+  <si>
+    <t>As a TA, I want to check all my application records and status to know the progress of my application.</t>
+  </si>
+  <si>
+    <t>As a TA, I want to upload a resume in plain text / Word format so that the course organizer can get a more complete picture of my abilities.</t>
+  </si>
+  <si>
+    <t>As a MO, I want to see all the TA information for my postings so that I can  review.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a MO, I want to mark individual applicants' applications as pass/fail so that I can complete application screening and sync status to TAs.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a TA / MO / Admin, I want to log in to the system with my account password so that I can access the user interface of the corresponding role.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a TA / MO / Admin, I want to use a smooth interface so that I can complete core operations to improve the user experience.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a TA, I want to withdraw my application with a status of "Under Review" so that I can re-select or modify my application.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a TA, I want to amend my profile information before submitting my application so that I can update my personal situation.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a TA, I want to filter positions based on criteria such as course name/available hours so that I can quickly find the right position.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a MO, I want to bulk tag the application status of multiple TAs so that I can improve the review process.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a MO, I want to see core data for all positions I post so that I can understand the progress of hiring.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a Admin, I want to see all MOs and TAs' personal information so that I can stay on top of the college-wide recruitment progress.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a Admin, I want to reset the MO/TA's password or delete an invalid so that I can maintain account security.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a TA / MO / Admin, I want to see pagination when there is too much list data so that I can improve the browsing experience.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a Admin, I want to record key actions and be able to view logs so that I can trace back to the history of operations.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a TA, I want to be alerted when my application status changes so that I can stay up to date with the outcome of my application.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a TA, I want to export my file information to JSON format so that I can backup offline.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a MO, I want to add specific skill requirements when posting a job so that I can match hiring needs procisely.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a MO, I want to fill out a comment at the time of review so that I can explain the reason for the review to the TA.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a MO, I want to look at TAs' past teaching assistant experiences so that it can help me assist in review decisions.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a Admin, I want to count the recruitment data of the whole college so that I can assist the college management decision-making.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a Admin, I want to export the core data of the whole hospital to CSV format so that it can be analysed offline.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a Admin, I want to restrict the MO from only operating the posts I post so that I can ensure data security.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a TA / MO / Admin, I want to use a more user-friendly interface so that it can improve the user experience.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a TA / MO / Admin, I want to switch between Chinese and English interfaces so that it can adapt to international usage scenarios.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a MO, I want to export the applicant information for this position in Excel format so that it can be viewed and statisticed offline offline.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a TA, I want to see a score on how well my skills match the position so that it can assist in job selection.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a MO, I want the system to automatically screen and prioritize high-match TAs so that it can improve screening efficiency.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a MO, I want the system to automatically extract resume core keywords so that I can quickly understand TA competencies.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a Admin, I want to get recommendations for optimizing TA assignments so that it can balance my workload.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a Admin, I want to get reference recommendations for the number of TA recruitments for each course/activity to assist in planning.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a Admin, I want to adjust the weight of job skill matching so that I can make the matching results more relevant to my actual needs.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>As a system user, I want to validate AI-generated results so that I can avoid logical errors.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1137,7 +1110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1244,6 +1217,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1264,104 +1243,7 @@
         <charset val="134"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FFFFFFFF"/>
-        <charset val="134"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF6495ED"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="18"/>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="微软雅黑"/>
-        <family val="2"/>
-        <charset val="134"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1404,6 +1286,22 @@
         <charset val="134"/>
         <scheme val="none"/>
       </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1419,6 +1317,36 @@
         <scheme val="none"/>
       </font>
       <alignment vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="18"/>
+        <name val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1463,6 +1391,57 @@
         <bottom/>
       </border>
     </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+        <charset val="134"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF6495ED"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1477,18 +1456,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ProductBacklogTable" displayName="ProductBacklogTable" ref="A1:J50" headerRowDxfId="3" dataDxfId="7" totalsRowDxfId="13" headerRowBorderDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ProductBacklogTable" displayName="ProductBacklogTable" ref="A1:J50" headerRowDxfId="13" dataDxfId="11" totalsRowDxfId="10" headerRowBorderDxfId="12">
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Story ID" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Story Name" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Priority" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Story ID" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Story Name" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Priority" dataDxfId="7"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Iteration (Sprint) number" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Acceptance Criteria" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Estimation/day" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Notes" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Date started (or planned)" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Date finished (or planned)" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Acceptance Criteria" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Estimation/day" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Notes" dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Date started (or planned)" dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Date finished (or planned)" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -1784,7 +1763,7 @@
   <sheetFormatPr defaultRowHeight="22.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.21875" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="44" style="4" customWidth="1"/>
+    <col min="2" max="2" width="44" style="32" customWidth="1"/>
     <col min="3" max="3" width="43.44140625" style="3" customWidth="1"/>
     <col min="4" max="4" width="11.21875" style="19" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="33.44140625" style="4" bestFit="1" customWidth="1"/>
@@ -1799,7 +1778,7 @@
       <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25" t="s">
+      <c r="B1" s="26" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="26" t="s">
@@ -1815,7 +1794,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="28" t="s">
-        <v>177</v>
+        <v>35</v>
       </c>
       <c r="H1" s="26" t="s">
         <v>6</v>
@@ -1831,70 +1810,70 @@
       <c r="A2" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="D2" s="23" t="s">
         <v>10</v>
-      </c>
-      <c r="C2" s="22" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="23" t="s">
-        <v>12</v>
       </c>
       <c r="E2" s="21">
         <v>1</v>
       </c>
       <c r="F2" s="22" t="s">
-        <v>13</v>
+        <v>155</v>
       </c>
       <c r="G2" s="20"/>
       <c r="H2" s="29" t="s">
-        <v>14</v>
+        <v>80</v>
       </c>
       <c r="I2" s="24"/>
       <c r="J2" s="24"/>
     </row>
     <row r="3" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>16</v>
+        <v>11</v>
+      </c>
+      <c r="B3" s="30" t="s">
+        <v>67</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>17</v>
+        <v>156</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E3" s="10">
         <v>1</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>18</v>
+        <v>157</v>
       </c>
       <c r="G3" s="9"/>
       <c r="H3" s="30"/>
       <c r="I3" s="12"/>
       <c r="J3" s="12"/>
     </row>
-    <row r="4" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" ht="167.4" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>20</v>
+        <v>12</v>
+      </c>
+      <c r="B4" s="31" t="s">
+        <v>68</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>21</v>
+        <v>190</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E4" s="5">
         <v>1</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>22</v>
+        <v>158</v>
       </c>
       <c r="G4" s="6"/>
       <c r="H4" s="31"/>
@@ -1903,22 +1882,22 @@
     </row>
     <row r="5" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>24</v>
+        <v>13</v>
+      </c>
+      <c r="B5" s="30" t="s">
+        <v>69</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>25</v>
+        <v>191</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E5" s="10">
         <v>1</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>26</v>
+        <v>159</v>
       </c>
       <c r="G5" s="9"/>
       <c r="H5" s="30"/>
@@ -1927,22 +1906,22 @@
     </row>
     <row r="6" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>28</v>
+        <v>14</v>
+      </c>
+      <c r="B6" s="31" t="s">
+        <v>70</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>29</v>
+        <v>181</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E6" s="5">
         <v>1</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>30</v>
+        <v>71</v>
       </c>
       <c r="G6" s="6"/>
       <c r="H6" s="31"/>
@@ -1951,22 +1930,22 @@
     </row>
     <row r="7" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>32</v>
+        <v>15</v>
+      </c>
+      <c r="B7" s="30" t="s">
+        <v>160</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>33</v>
+        <v>193</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E7" s="10">
         <v>1</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>34</v>
+        <v>161</v>
       </c>
       <c r="G7" s="9"/>
       <c r="H7" s="30"/>
@@ -1975,46 +1954,46 @@
     </row>
     <row r="8" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>36</v>
+        <v>16</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>72</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>37</v>
+        <v>194</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E8" s="5">
         <v>1</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>38</v>
+        <v>73</v>
       </c>
       <c r="G8" s="6"/>
       <c r="H8" s="31"/>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
     </row>
-    <row r="9" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" ht="165" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>40</v>
+        <v>17</v>
+      </c>
+      <c r="B9" s="30" t="s">
+        <v>74</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>223</v>
+        <v>195</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E9" s="10">
         <v>1</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>41</v>
+        <v>75</v>
       </c>
       <c r="G9" s="9"/>
       <c r="H9" s="30"/>
@@ -2023,22 +2002,22 @@
     </row>
     <row r="10" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>46</v>
+        <v>18</v>
+      </c>
+      <c r="B10" s="31" t="s">
+        <v>76</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>212</v>
+        <v>186</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E10" s="5">
         <v>1</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>47</v>
+        <v>77</v>
       </c>
       <c r="G10" s="6"/>
       <c r="H10" s="31"/>
@@ -2047,48 +2026,48 @@
     </row>
     <row r="11" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>49</v>
+        <v>19</v>
+      </c>
+      <c r="B11" s="30" t="s">
+        <v>78</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>213</v>
+        <v>196</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E11" s="10">
         <v>1</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>50</v>
+        <v>79</v>
       </c>
       <c r="G11" s="9"/>
       <c r="H11" s="30" t="s">
-        <v>51</v>
+        <v>81</v>
       </c>
       <c r="I11" s="12"/>
       <c r="J11" s="12"/>
     </row>
     <row r="12" spans="1:10" ht="130.19999999999999" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>60</v>
+        <v>41</v>
+      </c>
+      <c r="B12" s="31" t="s">
+        <v>82</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>61</v>
+        <v>197</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>187</v>
+        <v>42</v>
       </c>
       <c r="E12" s="5">
         <v>1</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>62</v>
+        <v>84</v>
       </c>
       <c r="G12" s="6"/>
       <c r="H12" s="31"/>
@@ -2097,22 +2076,22 @@
     </row>
     <row r="13" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>189</v>
+        <v>43</v>
+      </c>
+      <c r="B13" s="30" t="s">
+        <v>83</v>
       </c>
       <c r="C13" s="39" t="s">
-        <v>224</v>
+        <v>182</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>187</v>
+        <v>42</v>
       </c>
       <c r="E13" s="10">
         <v>1</v>
       </c>
-      <c r="F13" s="11" t="s">
-        <v>214</v>
+      <c r="F13" s="39" t="s">
+        <v>85</v>
       </c>
       <c r="G13" s="9"/>
       <c r="H13" s="30"/>
@@ -2121,22 +2100,22 @@
     </row>
     <row r="14" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>53</v>
+        <v>20</v>
+      </c>
+      <c r="B14" s="31" t="s">
+        <v>86</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>54</v>
+        <v>198</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="E14" s="5">
         <v>2</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>56</v>
+        <v>162</v>
       </c>
       <c r="G14" s="6"/>
       <c r="H14" s="31"/>
@@ -2145,22 +2124,22 @@
     </row>
     <row r="15" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>58</v>
+        <v>22</v>
+      </c>
+      <c r="B15" s="30" t="s">
+        <v>87</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>225</v>
+        <v>199</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="E15" s="10">
         <v>2</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="G15" s="9"/>
       <c r="H15" s="30"/>
@@ -2169,48 +2148,48 @@
     </row>
     <row r="16" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
-        <v>190</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>63</v>
+        <v>44</v>
+      </c>
+      <c r="B16" s="31" t="s">
+        <v>89</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>64</v>
+        <v>192</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="E16" s="5">
         <v>2</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>65</v>
+        <v>163</v>
       </c>
       <c r="G16" s="6"/>
       <c r="H16" s="31" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="I16" s="8"/>
       <c r="J16" s="8"/>
     </row>
     <row r="17" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="10" t="s">
-        <v>191</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>67</v>
+        <v>45</v>
+      </c>
+      <c r="B17" s="30" t="s">
+        <v>91</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>226</v>
+        <v>164</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="E17" s="10">
         <v>2</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>215</v>
+        <v>165</v>
       </c>
       <c r="G17" s="9"/>
       <c r="H17" s="30"/>
@@ -2219,22 +2198,22 @@
     </row>
     <row r="18" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
-        <v>192</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>216</v>
+        <v>46</v>
+      </c>
+      <c r="B18" s="40" t="s">
+        <v>92</v>
+      </c>
+      <c r="C18" s="41" t="s">
+        <v>183</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="E18" s="5">
         <v>2</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>185</v>
+        <v>93</v>
       </c>
       <c r="G18" s="6"/>
       <c r="H18" s="31"/>
@@ -2243,22 +2222,22 @@
     </row>
     <row r="19" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="10" t="s">
-        <v>193</v>
-      </c>
-      <c r="B19" s="10" t="s">
-        <v>68</v>
+        <v>47</v>
+      </c>
+      <c r="B19" s="30" t="s">
+        <v>166</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>69</v>
+        <v>184</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="E19" s="10">
         <v>2</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>70</v>
+        <v>167</v>
       </c>
       <c r="G19" s="9"/>
       <c r="H19" s="30"/>
@@ -2267,22 +2246,22 @@
     </row>
     <row r="20" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>71</v>
+        <v>48</v>
+      </c>
+      <c r="B20" s="31" t="s">
+        <v>94</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>72</v>
+        <v>200</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="E20" s="5">
         <v>2</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>73</v>
+        <v>168</v>
       </c>
       <c r="G20" s="6"/>
       <c r="H20" s="31"/>
@@ -2291,22 +2270,22 @@
     </row>
     <row r="21" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="10" t="s">
-        <v>195</v>
-      </c>
-      <c r="B21" s="10" t="s">
-        <v>77</v>
+        <v>49</v>
+      </c>
+      <c r="B21" s="30" t="s">
+        <v>95</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>78</v>
+        <v>201</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="E21" s="10">
         <v>2</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="G21" s="9"/>
       <c r="H21" s="30"/>
@@ -2315,22 +2294,22 @@
     </row>
     <row r="22" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>217</v>
+        <v>50</v>
+      </c>
+      <c r="B22" s="31" t="s">
+        <v>97</v>
+      </c>
+      <c r="C22" s="41" t="s">
+        <v>202</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="E22" s="5">
         <v>2</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>218</v>
+        <v>98</v>
       </c>
       <c r="G22" s="6"/>
       <c r="H22" s="31"/>
@@ -2339,22 +2318,22 @@
     </row>
     <row r="23" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="10" t="s">
-        <v>197</v>
-      </c>
-      <c r="B23" s="10" t="s">
-        <v>80</v>
+        <v>51</v>
+      </c>
+      <c r="B23" s="30" t="s">
+        <v>99</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>81</v>
+        <v>203</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="E23" s="10">
         <v>2</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="G23" s="9"/>
       <c r="H23" s="30"/>
@@ -2363,22 +2342,22 @@
     </row>
     <row r="24" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>219</v>
+        <v>38</v>
+      </c>
+      <c r="B24" s="31" t="s">
+        <v>101</v>
+      </c>
+      <c r="C24" s="41" t="s">
+        <v>204</v>
       </c>
       <c r="D24" s="16" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="E24" s="5">
         <v>2</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>88</v>
+        <v>102</v>
       </c>
       <c r="G24" s="6"/>
       <c r="H24" s="31"/>
@@ -2387,22 +2366,22 @@
     </row>
     <row r="25" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="10" t="s">
-        <v>198</v>
-      </c>
-      <c r="B25" s="10" t="s">
-        <v>89</v>
+        <v>52</v>
+      </c>
+      <c r="B25" s="30" t="s">
+        <v>103</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>90</v>
+        <v>205</v>
       </c>
       <c r="D25" s="16" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="E25" s="10">
         <v>2</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="G25" s="9"/>
       <c r="H25" s="30"/>
@@ -2411,48 +2390,46 @@
     </row>
     <row r="26" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>102</v>
+        <v>53</v>
+      </c>
+      <c r="B26" s="31" t="s">
+        <v>105</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>103</v>
+        <v>169</v>
       </c>
       <c r="D26" s="16" t="s">
-        <v>180</v>
+        <v>37</v>
       </c>
       <c r="E26" s="5">
         <v>2</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G26" s="6"/>
-      <c r="H26" s="31" t="s">
-        <v>220</v>
-      </c>
+      <c r="H26" s="31"/>
       <c r="I26" s="8"/>
       <c r="J26" s="8"/>
     </row>
     <row r="27" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="B27" s="10" t="s">
-        <v>93</v>
+        <v>23</v>
+      </c>
+      <c r="B27" s="30" t="s">
+        <v>107</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>94</v>
+        <v>170</v>
       </c>
       <c r="D27" s="17" t="s">
-        <v>95</v>
+        <v>24</v>
       </c>
       <c r="E27" s="10">
         <v>3</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>96</v>
+        <v>171</v>
       </c>
       <c r="G27" s="9"/>
       <c r="H27" s="30"/>
@@ -2461,74 +2438,74 @@
     </row>
     <row r="28" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>98</v>
+        <v>25</v>
+      </c>
+      <c r="B28" s="31" t="s">
+        <v>108</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>99</v>
+        <v>206</v>
       </c>
       <c r="D28" s="17" t="s">
-        <v>95</v>
+        <v>24</v>
       </c>
       <c r="E28" s="5">
         <v>3</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="G28" s="6"/>
       <c r="H28" s="31" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="I28" s="8"/>
       <c r="J28" s="8"/>
     </row>
     <row r="29" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="10" t="s">
-        <v>179</v>
-      </c>
-      <c r="B29" s="10" t="s">
-        <v>105</v>
+        <v>36</v>
+      </c>
+      <c r="B29" s="30" t="s">
+        <v>111</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>106</v>
+        <v>207</v>
       </c>
       <c r="D29" s="17" t="s">
-        <v>95</v>
+        <v>24</v>
       </c>
       <c r="E29" s="10">
         <v>3</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>107</v>
+        <v>172</v>
       </c>
       <c r="G29" s="9"/>
       <c r="H29" s="30" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="I29" s="12"/>
       <c r="J29" s="12"/>
     </row>
     <row r="30" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>109</v>
+        <v>54</v>
+      </c>
+      <c r="B30" s="31" t="s">
+        <v>113</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>110</v>
+        <v>208</v>
       </c>
       <c r="D30" s="17" t="s">
-        <v>95</v>
+        <v>24</v>
       </c>
       <c r="E30" s="5">
         <v>3</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="G30" s="6"/>
       <c r="H30" s="31"/>
@@ -2537,22 +2514,22 @@
     </row>
     <row r="31" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="10" t="s">
-        <v>201</v>
-      </c>
-      <c r="B31" s="10" t="s">
-        <v>112</v>
+        <v>55</v>
+      </c>
+      <c r="B31" s="30" t="s">
+        <v>115</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>113</v>
+        <v>209</v>
       </c>
       <c r="D31" s="17" t="s">
-        <v>95</v>
+        <v>24</v>
       </c>
       <c r="E31" s="10">
         <v>3</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="G31" s="9"/>
       <c r="H31" s="30"/>
@@ -2561,22 +2538,22 @@
     </row>
     <row r="32" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>115</v>
+        <v>56</v>
+      </c>
+      <c r="B32" s="31" t="s">
+        <v>117</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>116</v>
+        <v>185</v>
       </c>
       <c r="D32" s="17" t="s">
-        <v>95</v>
+        <v>24</v>
       </c>
       <c r="E32" s="5">
         <v>3</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G32" s="6"/>
       <c r="H32" s="31"/>
@@ -2585,22 +2562,22 @@
     </row>
     <row r="33" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="10" t="s">
-        <v>203</v>
-      </c>
-      <c r="B33" s="10" t="s">
-        <v>118</v>
+        <v>57</v>
+      </c>
+      <c r="B33" s="30" t="s">
+        <v>119</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>119</v>
+        <v>210</v>
       </c>
       <c r="D33" s="17" t="s">
-        <v>95</v>
+        <v>24</v>
       </c>
       <c r="E33" s="10">
         <v>3</v>
       </c>
       <c r="F33" s="11" t="s">
-        <v>120</v>
+        <v>173</v>
       </c>
       <c r="G33" s="9"/>
       <c r="H33" s="30"/>
@@ -2609,22 +2586,22 @@
     </row>
     <row r="34" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
-        <v>204</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>121</v>
+        <v>58</v>
+      </c>
+      <c r="B34" s="31" t="s">
+        <v>120</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>122</v>
+        <v>187</v>
       </c>
       <c r="D34" s="17" t="s">
-        <v>95</v>
+        <v>24</v>
       </c>
       <c r="E34" s="5">
         <v>3</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="G34" s="6"/>
       <c r="H34" s="31"/>
@@ -2633,22 +2610,22 @@
     </row>
     <row r="35" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="10" t="s">
-        <v>205</v>
-      </c>
-      <c r="B35" s="10" t="s">
-        <v>124</v>
+        <v>59</v>
+      </c>
+      <c r="B35" s="30" t="s">
+        <v>122</v>
       </c>
       <c r="C35" s="11" t="s">
-        <v>125</v>
+        <v>211</v>
       </c>
       <c r="D35" s="17" t="s">
-        <v>95</v>
+        <v>24</v>
       </c>
       <c r="E35" s="10">
         <v>3</v>
       </c>
       <c r="F35" s="11" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="G35" s="9"/>
       <c r="H35" s="30"/>
@@ -2657,48 +2634,48 @@
     </row>
     <row r="36" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
-        <v>206</v>
-      </c>
-      <c r="B36" s="5" t="s">
-        <v>127</v>
+        <v>60</v>
+      </c>
+      <c r="B36" s="31" t="s">
+        <v>124</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>128</v>
+        <v>212</v>
       </c>
       <c r="D36" s="17" t="s">
-        <v>95</v>
+        <v>24</v>
       </c>
       <c r="E36" s="5">
         <v>3</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="G36" s="6"/>
       <c r="H36" s="31" t="s">
-        <v>176</v>
+        <v>126</v>
       </c>
       <c r="I36" s="8"/>
       <c r="J36" s="8"/>
     </row>
     <row r="37" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="10" t="s">
-        <v>207</v>
-      </c>
-      <c r="B37" s="10" t="s">
-        <v>130</v>
+        <v>61</v>
+      </c>
+      <c r="B37" s="30" t="s">
+        <v>127</v>
       </c>
       <c r="C37" s="11" t="s">
-        <v>131</v>
+        <v>213</v>
       </c>
       <c r="D37" s="17" t="s">
-        <v>95</v>
+        <v>24</v>
       </c>
       <c r="E37" s="10">
         <v>3</v>
       </c>
       <c r="F37" s="11" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="G37" s="9"/>
       <c r="H37" s="30"/>
@@ -2707,22 +2684,22 @@
     </row>
     <row r="38" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="B38" s="5" t="s">
-        <v>133</v>
+        <v>62</v>
+      </c>
+      <c r="B38" s="31" t="s">
+        <v>129</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>134</v>
+        <v>188</v>
       </c>
       <c r="D38" s="17" t="s">
-        <v>95</v>
+        <v>24</v>
       </c>
       <c r="E38" s="5">
         <v>3</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="G38" s="6"/>
       <c r="H38" s="31"/>
@@ -2731,22 +2708,22 @@
     </row>
     <row r="39" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="10" t="s">
-        <v>209</v>
-      </c>
-      <c r="B39" s="10" t="s">
-        <v>136</v>
+        <v>63</v>
+      </c>
+      <c r="B39" s="30" t="s">
+        <v>131</v>
       </c>
       <c r="C39" s="11" t="s">
-        <v>137</v>
+        <v>214</v>
       </c>
       <c r="D39" s="17" t="s">
-        <v>95</v>
+        <v>24</v>
       </c>
       <c r="E39" s="10">
         <v>3</v>
       </c>
       <c r="F39" s="11" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="G39" s="9"/>
       <c r="H39" s="30"/>
@@ -2755,22 +2732,22 @@
     </row>
     <row r="40" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="B40" s="5" t="s">
-        <v>139</v>
+        <v>64</v>
+      </c>
+      <c r="B40" s="31" t="s">
+        <v>133</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>140</v>
+        <v>215</v>
       </c>
       <c r="D40" s="17" t="s">
-        <v>95</v>
+        <v>24</v>
       </c>
       <c r="E40" s="5">
         <v>3</v>
       </c>
       <c r="F40" s="7" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="G40" s="6"/>
       <c r="H40" s="31"/>
@@ -2779,100 +2756,96 @@
     </row>
     <row r="41" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="B41" s="10" t="s">
-        <v>84</v>
+        <v>65</v>
+      </c>
+      <c r="B41" s="30" t="s">
+        <v>135</v>
       </c>
       <c r="C41" s="11" t="s">
-        <v>85</v>
+        <v>174</v>
       </c>
       <c r="D41" s="17" t="s">
-        <v>183</v>
+        <v>40</v>
       </c>
       <c r="E41" s="10">
         <v>3</v>
       </c>
       <c r="F41" s="11" t="s">
-        <v>86</v>
+        <v>136</v>
       </c>
       <c r="G41" s="9"/>
-      <c r="H41" s="30" t="s">
-        <v>221</v>
-      </c>
+      <c r="H41" s="30"/>
       <c r="I41" s="12"/>
       <c r="J41" s="12"/>
     </row>
     <row r="42" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="B42" s="5" t="s">
-        <v>74</v>
+        <v>39</v>
+      </c>
+      <c r="B42" s="31" t="s">
+        <v>175</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>75</v>
+        <v>216</v>
       </c>
       <c r="D42" s="17" t="s">
-        <v>183</v>
+        <v>40</v>
       </c>
       <c r="E42" s="5">
         <v>3</v>
       </c>
       <c r="F42" s="7" t="s">
-        <v>76</v>
+        <v>176</v>
       </c>
       <c r="G42" s="6"/>
-      <c r="H42" s="31" t="s">
-        <v>222</v>
-      </c>
+      <c r="H42" s="31"/>
       <c r="I42" s="8"/>
       <c r="J42" s="8"/>
     </row>
     <row r="43" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="B43" s="10" t="s">
-        <v>143</v>
+        <v>26</v>
+      </c>
+      <c r="B43" s="30" t="s">
+        <v>137</v>
       </c>
       <c r="C43" s="11" t="s">
-        <v>144</v>
+        <v>217</v>
       </c>
       <c r="D43" s="18" t="s">
-        <v>145</v>
+        <v>27</v>
       </c>
       <c r="E43" s="10">
         <v>4</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>146</v>
+        <v>177</v>
       </c>
       <c r="G43" s="9"/>
       <c r="H43" s="30" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="I43" s="12"/>
       <c r="J43" s="12"/>
     </row>
     <row r="44" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="B44" s="5" t="s">
-        <v>149</v>
+        <v>28</v>
+      </c>
+      <c r="B44" s="31" t="s">
+        <v>139</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>150</v>
+        <v>178</v>
       </c>
       <c r="D44" s="18" t="s">
-        <v>145</v>
+        <v>27</v>
       </c>
       <c r="E44" s="5">
         <v>4</v>
       </c>
       <c r="F44" s="7" t="s">
-        <v>151</v>
+        <v>140</v>
       </c>
       <c r="G44" s="6"/>
       <c r="H44" s="31"/>
@@ -2881,22 +2854,22 @@
     </row>
     <row r="45" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="B45" s="10" t="s">
-        <v>153</v>
+        <v>29</v>
+      </c>
+      <c r="B45" s="30" t="s">
+        <v>179</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>154</v>
+        <v>218</v>
       </c>
       <c r="D45" s="18" t="s">
-        <v>145</v>
+        <v>27</v>
       </c>
       <c r="E45" s="10">
         <v>4</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>155</v>
+        <v>180</v>
       </c>
       <c r="G45" s="9"/>
       <c r="H45" s="30"/>
@@ -2905,22 +2878,22 @@
     </row>
     <row r="46" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="B46" s="5" t="s">
-        <v>157</v>
+        <v>30</v>
+      </c>
+      <c r="B46" s="31" t="s">
+        <v>141</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>158</v>
+        <v>219</v>
       </c>
       <c r="D46" s="18" t="s">
-        <v>145</v>
+        <v>27</v>
       </c>
       <c r="E46" s="5">
         <v>4</v>
       </c>
       <c r="F46" s="7" t="s">
-        <v>159</v>
+        <v>142</v>
       </c>
       <c r="G46" s="6"/>
       <c r="H46" s="31"/>
@@ -2929,22 +2902,22 @@
     </row>
     <row r="47" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="10" t="s">
-        <v>160</v>
-      </c>
-      <c r="B47" s="10" t="s">
-        <v>161</v>
+        <v>31</v>
+      </c>
+      <c r="B47" s="30" t="s">
+        <v>143</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>162</v>
+        <v>220</v>
       </c>
       <c r="D47" s="18" t="s">
-        <v>145</v>
+        <v>27</v>
       </c>
       <c r="E47" s="10">
         <v>4</v>
       </c>
       <c r="F47" s="11" t="s">
-        <v>163</v>
+        <v>144</v>
       </c>
       <c r="G47" s="9"/>
       <c r="H47" s="30"/>
@@ -2953,22 +2926,22 @@
     </row>
     <row r="48" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="B48" s="5" t="s">
-        <v>165</v>
+        <v>32</v>
+      </c>
+      <c r="B48" s="31" t="s">
+        <v>145</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>166</v>
+        <v>221</v>
       </c>
       <c r="D48" s="18" t="s">
-        <v>145</v>
+        <v>27</v>
       </c>
       <c r="E48" s="5">
         <v>4</v>
       </c>
       <c r="F48" s="7" t="s">
-        <v>167</v>
+        <v>146</v>
       </c>
       <c r="G48" s="6"/>
       <c r="H48" s="31"/>
@@ -2977,22 +2950,22 @@
     </row>
     <row r="49" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="10" t="s">
-        <v>168</v>
-      </c>
-      <c r="B49" s="10" t="s">
-        <v>169</v>
+        <v>33</v>
+      </c>
+      <c r="B49" s="30" t="s">
+        <v>147</v>
       </c>
       <c r="C49" s="11" t="s">
-        <v>170</v>
+        <v>222</v>
       </c>
       <c r="D49" s="18" t="s">
-        <v>145</v>
+        <v>27</v>
       </c>
       <c r="E49" s="10">
         <v>4</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>171</v>
+        <v>148</v>
       </c>
       <c r="G49" s="9"/>
       <c r="H49" s="30"/>
@@ -3001,42 +2974,42 @@
     </row>
     <row r="50" spans="1:10" ht="130.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="B50" s="5" t="s">
-        <v>173</v>
+        <v>34</v>
+      </c>
+      <c r="B50" s="31" t="s">
+        <v>149</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>174</v>
+        <v>223</v>
       </c>
       <c r="D50" s="18" t="s">
-        <v>145</v>
+        <v>27</v>
       </c>
       <c r="E50" s="5">
         <v>4</v>
       </c>
       <c r="F50" s="7" t="s">
-        <v>175</v>
+        <v>150</v>
       </c>
       <c r="G50" s="6"/>
       <c r="H50" s="31"/>
       <c r="I50" s="8"/>
       <c r="J50" s="8"/>
     </row>
-    <row r="51" spans="1:10" s="1" customFormat="1" ht="43.2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" s="1" customFormat="1" ht="94.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="33" t="s">
-        <v>178</v>
-      </c>
-      <c r="B51" s="33" t="s">
-        <v>42</v>
+        <v>151</v>
+      </c>
+      <c r="B51" s="37" t="s">
+        <v>152</v>
       </c>
       <c r="C51" s="34" t="s">
-        <v>43</v>
+        <v>153</v>
       </c>
       <c r="D51" s="35"/>
       <c r="E51" s="33"/>
       <c r="F51" s="34" t="s">
-        <v>44</v>
+        <v>154</v>
       </c>
       <c r="G51" s="36"/>
       <c r="H51" s="37"/>

</xml_diff>